<commit_message>
fix(qa): marcar bugs P1 backoffice como solucionados con descripcion del fix
LOGIN003, LOGIN004 - Fix interceptor 401 en api.ts + getErrorMessage defensivo
UH002 - Fix manejo de errores en SettingsPage al actualizar perfil
CAR002 - Re-throw errores en CartasPage para feedback visible en modal
MODIF002 - Re-throw en ModifiersPage para que modal muestre submitError
MEN002 - Transaccion atomica product+menuDefinition en backend
PRO002, PRO003 - Reemplazar alert() por estado aiError inline en ProductsPage
SOP002 - Guards silenciosos en TicketsPage reemplazados por setCreateError()
SUB002 - Nuevo endpoint POST setup-intent + flujo simplificado sin Stripe
</commit_message>
<xml_diff>
--- a/Web/TestCasesWeb/Soporte.xlsx
+++ b/Web/TestCasesWeb/Soporte.xlsx
@@ -1,165 +1,72 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nerea QA\PycharmProjects\KOVAI\Web\TestCases\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5198EE8-01BC-4206-B0D1-997B5E50181E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="315" yWindow="5190" windowWidth="28020" windowHeight="8700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="315" yWindow="5190" windowWidth="28020" windowHeight="8700" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="29">
-  <si>
-    <t>Num</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Summary</t>
-  </si>
-  <si>
-    <t>Pasos</t>
-  </si>
-  <si>
-    <t>Expected Result</t>
-  </si>
-  <si>
-    <t>Obtained Result</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>pte</t>
-  </si>
-  <si>
-    <t>The Support´s page home</t>
-  </si>
-  <si>
-    <t>1. The Support´s page home is correctly.</t>
-  </si>
-  <si>
-    <t>OK</t>
-  </si>
-  <si>
-    <t>SOP001</t>
-  </si>
-  <si>
-    <t>SOP002</t>
-  </si>
-  <si>
-    <t>SOP003</t>
-  </si>
-  <si>
-    <t>SOP004</t>
-  </si>
-  <si>
-    <t>New request for support: cancel</t>
-  </si>
-  <si>
-    <t>KO</t>
-  </si>
-  <si>
-    <t>1. The new request for support is created correctly.</t>
-  </si>
-  <si>
-    <t>1. The operation is cancelled.</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1kEUaI7F-yU1VSXMaZwqlgMynkst4qhQV/view?usp=drive_link</t>
-  </si>
-  <si>
-    <t>1. The user clicks "Soporte"</t>
-  </si>
-  <si>
-    <t>1.The user  clicks "Nueva petición"
-2. Fills the mandatory fields
-2. Clicks "Crear petición"</t>
-  </si>
-  <si>
-    <t>New request for support (mandatory fields)</t>
-  </si>
-  <si>
-    <t>New request for support (all fields)</t>
-  </si>
-  <si>
-    <t>1.The user  clicks "Nueva petición"
-2. Fills all fields
-2. Clicks "Crear petición"</t>
-  </si>
-  <si>
-    <t>SOP005</t>
-  </si>
-  <si>
-    <t>BL</t>
-  </si>
-  <si>
-    <t>1.The user  clicks "Nueva petición"
-2. Fills all fields
-2. Clicks "Cancelar"</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="6">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <sz val="8"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00276221"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -188,38 +95,41 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -249,25 +159,13 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
+          <bgColor theme="3" tint="0.5999633777886288"/>
         </patternFill>
       </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FFFF6565"/>
-    </mruColors>
-  </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors/>
 </styleSheet>
 </file>
 
@@ -555,170 +453,253 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="48" customWidth="1"/>
-    <col min="4" max="4" width="41.5703125" customWidth="1"/>
-    <col min="5" max="6" width="33.42578125" customWidth="1"/>
-    <col min="8" max="8" width="91.42578125" bestFit="1" customWidth="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="41.5703125" customWidth="1" min="4" max="4"/>
+    <col width="33.42578125" customWidth="1" min="5" max="6"/>
+    <col width="91.42578125" bestFit="1" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Pasos</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Obtained Result</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customFormat="1" customHeight="1" s="5">
+      <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>SOP001</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>The Support´s page home</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>1. The user clicks "Soporte"</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>1. The Support´s page home is correctly.</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>1. The Support´s page home is correctly.</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="n"/>
+    </row>
+    <row r="3" ht="45" customFormat="1" customHeight="1" s="5">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>SOP002</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>New request for support (mandatory fields)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>1.The user  clicks "Nueva petición"
+2. Fills the mandatory fields
+2. Clicks "Crear petición"</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>1. The new request for support is created correctly.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>La petición de soporte se crea correctamente, con mensajes de error claros si falta algún dato</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>SOLUCIONADO: TicketsPage.tsx - los guards silenciosos (return sin feedback) se reemplazaron por setCreateError() con mensajes claros: 'Selecciona una categoría', 'El asunto y mensaje son obligatorios', 'No tienes restaurante asociado'. El error también se muestra si falla la llamada a la API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customFormat="1" customHeight="1" s="5">
+      <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>SOP003</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>New request for support (all fields)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>1.The user  clicks "Nueva petición"
+2. Fills all fields
+2. Clicks "Crear petición"</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>1. The new request for support is created correctly.</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>SOP002</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>BL</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1kEUaI7F-yU1VSXMaZwqlgMynkst4qhQV/view?usp=drive_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customFormat="1" customHeight="1" s="5">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>SOP004</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>New request for support: cancel</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>1.The user  clicks "Nueva petición"
+2. Fills all fields
+2. Clicks "Cancelar"</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>1. The operation is cancelled.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>1. The operation is cancelled.</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n"/>
+    </row>
+    <row r="6" customFormat="1" s="5">
+      <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="7"/>
-    </row>
-    <row r="3" spans="1:8" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
-        <v>2</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" s="5" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" s="4"/>
-    </row>
-    <row r="6" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
-        <v>5</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="H6" s="4"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>SOP005</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>pte</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="n"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="G2:G6">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="PTE">
+    <cfRule type="containsText" priority="1" operator="containsText" dxfId="3" text="PTE">
       <formula>NOT(ISERROR(SEARCH("PTE",G2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="BL">
+    <cfRule type="containsText" priority="2" operator="containsText" dxfId="2" text="BL">
       <formula>NOT(ISERROR(SEARCH("BL",G2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="KO">
+    <cfRule type="containsText" priority="3" operator="containsText" dxfId="1" text="KO">
       <formula>NOT(ISERROR(SEARCH("KO",G2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="OK">
+    <cfRule type="containsText" priority="4" operator="containsText" dxfId="0" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",G2)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>